<commit_message>
Fixed link to slides.
</commit_message>
<xml_diff>
--- a/Schedule.xlsx
+++ b/Schedule.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jbryer/SPS Dropbox/Jason Bryer/Teaching/DATA606 2025 Spring/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96BF60A3-F2BB-CA42-9310-B74DC92940AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F6C5430-9992-284D-8263-558806553813}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1680" yWindow="10920" windowWidth="19700" windowHeight="15960" xr2:uid="{A772458D-4E7B-8249-8B6B-34FE7D5BD316}"/>
   </bookViews>
@@ -292,10 +292,10 @@
     <t>NlJwU7-u1lo</t>
   </si>
   <si>
-    <t>06-Infernce_for_Categorial_Data</t>
-  </si>
-  <si>
     <t>AsTAHYMIXkc</t>
+  </si>
+  <si>
+    <t>06-Inference_for_Categorical_Data</t>
   </si>
 </sst>
 </file>
@@ -937,10 +937,10 @@
         <v>53</v>
       </c>
       <c r="F10" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="G10" t="s">
         <v>86</v>
-      </c>
-      <c r="G10" t="s">
-        <v>85</v>
       </c>
       <c r="H10" s="4"/>
     </row>

</xml_diff>